<commit_message>
Monkole capacités : 104 lits réels répartis par unité, taux d'occupation par unité
- Lits CHME : chirurgie 13, gynéco-obstétrique 27, médecine interne 15, néonatologie 12, pédiatrie 13,
  urgences 5, soins intensifs pédiatriques 12, réanimation 7 ; la capacité du CHME est leur total.
- Taux d'occupation moyen et du dernier jour par unité (CHME, Dashboard, résumé), avec couleurs d'alerte.
- L'ancienne répartition (lits des logiciels, fictifs inclus) est remplacée automatiquement dans le référentiel.
- Notez bien : taux d'unité au-delà de 100 %, relais de spécialités dans un même cabinet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NviAxNSL5tDnEBmBNdUMNs
</commit_message>
<xml_diff>
--- a/outils/monkole_capacites/Referentiel_Monkole.xlsx
+++ b/outils/monkole_capacites/Referentiel_Monkole.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -505,30 +505,20 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Lits réels CHME</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>104</v>
+          <t>Alerte : utilisation basse sous (ex. 0,50 = 50 %)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Alerte : utilisation basse sous (ex. 0,50 = 50 %)</t>
+          <t>Alerte : utilisation haute à partir de (ex. 0,85 = 85 %)</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Alerte : utilisation haute à partir de (ex. 0,85 = 85 %)</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
         <v>0.85</v>
       </c>
     </row>
@@ -553,7 +543,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Lits par unité tels que paramétrés dans les logiciels (indicatif). La capacité réelle est dans Paramètres.</t>
+          <t>Lits réels par unité (libellés Hospi CHIR, Hospi GO...). Leur total est la capacité du CHME.</t>
         </is>
       </c>
     </row>
@@ -576,7 +566,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -586,7 +576,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>54</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
@@ -596,7 +586,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -606,7 +596,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
@@ -626,7 +616,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -636,7 +626,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10">
@@ -646,7 +636,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monkole capacités : 104 lits réels répartis par unité, occupation par unité (#49)
- Lits CHME : chirurgie 13, gynéco-obstétrique 27, médecine interne 15, néonatologie 12, pédiatrie 13,
  urgences 5, soins intensifs pédiatriques 12, réanimation 7 ; la capacité du CHME est leur total.
- Taux d'occupation moyen et du dernier jour par unité (CHME, Dashboard, résumé), avec couleurs d'alerte.
- L'ancienne répartition (lits des logiciels, fictifs inclus) est remplacée automatiquement dans le référentiel.
- Notez bien : taux d'unité au-delà de 100 %, relais de spécialités dans un même cabinet.


Claude-Session: https://claude.ai/code/session_01NviAxNSL5tDnEBmBNdUMNs

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outils/monkole_capacites/Referentiel_Monkole.xlsx
+++ b/outils/monkole_capacites/Referentiel_Monkole.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -505,30 +505,20 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Lits réels CHME</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>104</v>
+          <t>Alerte : utilisation basse sous (ex. 0,50 = 50 %)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Alerte : utilisation basse sous (ex. 0,50 = 50 %)</t>
+          <t>Alerte : utilisation haute à partir de (ex. 0,85 = 85 %)</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Alerte : utilisation haute à partir de (ex. 0,85 = 85 %)</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
         <v>0.85</v>
       </c>
     </row>
@@ -553,7 +543,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Lits par unité tels que paramétrés dans les logiciels (indicatif). La capacité réelle est dans Paramètres.</t>
+          <t>Lits réels par unité (libellés Hospi CHIR, Hospi GO...). Leur total est la capacité du CHME.</t>
         </is>
       </c>
     </row>
@@ -576,7 +566,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -586,7 +576,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>54</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
@@ -596,7 +586,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -606,7 +596,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
@@ -626,7 +616,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -636,7 +626,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10">
@@ -646,7 +636,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monkole : 1 170 formulations du 01-28/09 classées dans le dictionnaire ; sorties Evolucare proposées à 4 jours
Diagnostics
- Dictionnaire_Diagnostics.xlsx : 1 170 formulations nouvelles classées (codes et statuts, « à valider »),
  38 diagnostics regroupés ajoutés (brûlure, bronchiolite, HTA gravidique, RCIU, cirrhose, cancer colorectal,
  trouble du rythme, psychose, dent incluse...). 2 727 formulations, 437 diagnostics regroupés.

Capacités
- Evolucare propose une sortie à 4 jours dès l'admission : une sortie à exactement 4 jours est une proposition
  (non comptée comme sortie réalisée ni dans la DMS), les autres dates sont réelles. Durée paramétrable dans le
  référentiel ; colonne « Sortie proposée » dans la base des hospitalisations ; textes mis à jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NviAxNSL5tDnEBmBNdUMNs
</commit_message>
<xml_diff>
--- a/outils/monkole_capacites/Referentiel_Monkole.xlsx
+++ b/outils/monkole_capacites/Referentiel_Monkole.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -531,6 +531,16 @@
       </c>
       <c r="B9" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Evolucare : durée de séjour proposée à l'admission (jours ; cette durée exacte = sortie non confirmée)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monkole : formulations du 01-28/09 classées ; sorties Evolucare proposées à 4 jours (#53)
Diagnostics
- Dictionnaire_Diagnostics.xlsx : 1 170 formulations nouvelles classées (codes et statuts, « à valider »),
  38 diagnostics regroupés ajoutés (brûlure, bronchiolite, HTA gravidique, RCIU, cirrhose, cancer colorectal,
  trouble du rythme, psychose, dent incluse...). 2 727 formulations, 437 diagnostics regroupés.

Capacités
- Evolucare propose une sortie à 4 jours dès l'admission : une sortie à exactement 4 jours est une proposition
  (non comptée comme sortie réalisée ni dans la DMS), les autres dates sont réelles. Durée paramétrable dans le
  référentiel ; colonne « Sortie proposée » dans la base des hospitalisations ; textes mis à jour.


Claude-Session: https://claude.ai/code/session_01NviAxNSL5tDnEBmBNdUMNs

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outils/monkole_capacites/Referentiel_Monkole.xlsx
+++ b/outils/monkole_capacites/Referentiel_Monkole.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -531,6 +531,16 @@
       </c>
       <c r="B9" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Evolucare : durée de séjour proposée à l'admission (jours ; cette durée exacte = sortie non confirmée)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>